<commit_message>
update bill page -5560922286
</commit_message>
<xml_diff>
--- a/bills/JXZFSP01/-5560922286/a04009deb7e69570bc9f5ca765210e487e41c38d8e120e2341bfe7056a39f72d/bill-2026-09-15.xlsx
+++ b/bills/JXZFSP01/-5560922286/a04009deb7e69570bc9f5ca765210e487e41c38d8e120e2341bfe7056a39f72d/bill-2026-09-15.xlsx
@@ -202,83 +202,110 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>09/15 13:31:22</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>24599</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>jxxiaomei521</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>09/15 11:35:25</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>688</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>tiantiananxin</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>总计</t>
-        </is>
-      </c>
-    </row>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>总入款</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>220000</t>
+          <t>总计</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>应下发</t>
+          <t>总入款</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>25287.36</t>
+          <t>220000</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>已下发</t>
+          <t>应下发</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>688</t>
+          <t>25287.36</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>已下发</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>25287</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>未下发</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>24599.36</t>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0.36</t>
         </is>
       </c>
     </row>

</xml_diff>